<commit_message>
Update P2_Form_Professional_Report_JuniorPlus_Table.xlsx with new data and formatting changes.
</commit_message>
<xml_diff>
--- a/P2_Form_Professional_Report_JuniorPlus_Table.xlsx
+++ b/P2_Form_Professional_Report_JuniorPlus_Table.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\CONG VIEC\project-management\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33D3FDED-AB3D-4365-A6BB-600A38BD5D4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E55BE52-D75F-4EBF-87B4-1E34EA32A4A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary_Ranking" sheetId="1" r:id="rId1"/>
+    <sheet name="Summary_Ranking" sheetId="1" state="hidden" r:id="rId1"/>
     <sheet name="Product_Engineer" sheetId="2" r:id="rId2"/>
-    <sheet name="Cấp độ năng lực theo vai trò" sheetId="3" r:id="rId3"/>
+    <sheet name="MÔ TẢ - PHỤ LỤC" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -193,9 +193,6 @@
     <t>Ứng viên lên track Senior/Lead; giao ownership dự án / mentor người khác.</t>
   </si>
   <si>
-    <t>CẤP ĐỘ NĂNG LỰC (THEO VAI TRÒ)</t>
-  </si>
-  <si>
     <t>Backend</t>
   </si>
   <si>
@@ -214,160 +211,163 @@
     <t>Thiết kế kiến trúc/module gọn; cải thiện performance/security; tests chắc; nâng chất lượng qua review.</t>
   </si>
   <si>
-    <t>Định hướng backend; ngăn lỗi hệ thống; mentoring đội; dẫn dắt refactor/migrations lớn an toàn.</t>
-  </si>
-  <si>
-    <t>Bàn giao ổn định; tách công việc thành tickets; chịu trách nhiệm bug đến khi đóng; báo risk sớm.</t>
-  </si>
-  <si>
     <t>C. DevOps &amp; vận hành</t>
   </si>
   <si>
-    <t>Dùng CI/CD; hiểu env/secrets; logging/error tracking; tham gia oncall/bugfix.</t>
-  </si>
-  <si>
-    <t>Cải thiện CI/CD (cache, gates); thêm metrics/alerts; rollback; cải thiện reliability &amp; MTTR.</t>
-  </si>
-  <si>
-    <t>Chuẩn hóa release/observability; playbooks; dẫn postmortem; mentoring thực hành ops.</t>
-  </si>
-  <si>
     <t>D. AI Agent &amp; cải tiến</t>
   </si>
   <si>
-    <t>Dùng AI Agent cho scaffolding/refactor/tests/debug; kỹ thuật prompt; review cẩn thận.</t>
-  </si>
-  <si>
-    <t>Prompt/workflow tái sử dụng; AI cho review &amp; debugging; đo impact (cycle thời gian/defects).</t>
-  </si>
-  <si>
-    <t>Dẫn dắt thực hành kỹ thuật AI; đào tạo đội; tự động hóa công việc lặp an toàn có governance.</t>
-  </si>
-  <si>
     <t>Designer</t>
   </si>
   <si>
-    <t>Tự giao UX flows &amp; UI specs; hình ảnh nhất quán; handoff rõ (states, spacing, tokens).</t>
-  </si>
-  <si>
-    <t>Cải thiện khả năng sử dụng qua research/heuristics; mở rộng design hệ thống; giảm rework với specs tốt hơn.</t>
-  </si>
-  <si>
-    <t>Định hướng design; tác động UX đo được; governance design hệ thống; mentoring cross-đội.</t>
-  </si>
-  <si>
-    <t>Bàn giao ổn định; scope rõ; lặp kịp thời; align ràng buộc với BE/FE sớm.</t>
-  </si>
-  <si>
-    <t>Quản lý đánh đổi; chuẩn bị variants; ghi chú quyết định; giảm rework qua review.</t>
-  </si>
-  <si>
-    <t>Nâng chuẩn bàn giao design (DoD, review checklist); gỡ block cross-đội; tính dự báo.</t>
-  </si>
-  <si>
-    <t>Làm việc với preview/staging; dùng tokens/components; specs phù hợp build consđào tạots.</t>
-  </si>
-  <si>
-    <t>Thúc đẩy áp dụng tokens/components; cải thiện handoff automation; giảm lỗi tích hợp &amp; rework.</t>
-  </si>
-  <si>
-    <t>Dẫn chuẩn hóa workflow design-to-dev với FE; playbooks và best thực hành.</t>
-  </si>
-  <si>
-    <t>AI cho wireframes, UX copy, variants; kỹ thuật prompt; validate với hệ thống consđào tạots.</t>
-  </si>
-  <si>
-    <t>Thư viện prompt tái sử dụng; đẩy nhanh research synthesis; đo impact lên cycle thời gian/rework.</t>
-  </si>
-  <si>
-    <t>Dẫn dắt thực hành design AI; đào tạo đội; tự động hóa công việc lặp an toàn; governance.</t>
-  </si>
-  <si>
     <t>FrontEnd</t>
   </si>
   <si>
-    <t>Tự triển khai tính năng (UI + state + tích hợp API); xử lý trường hợp lỗi không mong muốn xảy ra; code dễ bảo trì.</t>
-  </si>
-  <si>
-    <t>Cải thiện performance (bundle/render), accessibility; components tái sử dụng; kiến trúc/tests mạnh hơn.</t>
-  </si>
-  <si>
-    <t>Định hướng FE; dẫn refactor/design hệ thống; mentoring đội; ngăn lỗi UI hệ thống.</t>
-  </si>
-  <si>
-    <t>Bàn giao ổn định; chịu trách nhiệm bug; phối hợp BE/Designer; báo risk sớm.</t>
-  </si>
-  <si>
-    <t>Quản lý đánh đổi UX; giảm rework; nâng chất lượng qua specs, demos, tài liệu.</t>
-  </si>
-  <si>
-    <t>Nâng chuẩn bàn giao (component chuẩn, review checklist); gỡ block cross-đội; tính dự báo.</t>
-  </si>
-  <si>
-    <t>Dùng CI thành thạo; quản lý env/config; giám sát client errors; giữ build gọn.</t>
-  </si>
-  <si>
-    <t>Tối ưu CI (cache/gates); cải thiện build speed &amp; bundle size; rollback; reliability.</t>
-  </si>
-  <si>
-    <t>Chuẩn hóa release/observability FE; playbooks; mentoring đội; giảm client error/MTTR.</t>
-  </si>
-  <si>
-    <t>AI Agent để scaffold/refactor/tests/debug; kỹ thuật prompt; review cẩn thận.</t>
-  </si>
-  <si>
-    <t>Template prompt tái sử dụng (component/a11y/test); AI cho review/refactor; đo lường kết quả.</t>
-  </si>
-  <si>
-    <t>Dẫn dắt thực hành FE hỗ trợ AI; đào tạo đội; tự động hóa nhiệm vụ UI lặp an toàn.</t>
-  </si>
-  <si>
     <t>FullStack</t>
   </si>
   <si>
-    <t>Tự triển khai end-to-end (API+DB+UI); giữ chất lượng; tests cơ bản; xử lý trường hợp lỗi không mong muốn xảy ra.</t>
-  </si>
-  <si>
-    <t>Ranh giới BE/FE rõ; cải thiện perf/security; refactor an toàn; tests mạnh.</t>
-  </si>
-  <si>
-    <t>Định hướng end-to-end; ngăn lỗi hệ thống; mentoring đội; dẫn refactor/migrations lớn.</t>
-  </si>
-  <si>
-    <t>Chịu trách nhiệm tính năng end-to-end; ổn định; báo risk sớm; sửa đến khi xong.</t>
-  </si>
-  <si>
-    <t>Quản lý scope/risk; đàm phán đánh đổi; giảm rework; cải thiện docs/handoff.</t>
-  </si>
-  <si>
-    <t>Cải thiện tính dự báo; định nghĩa chuẩn (DoD, review checklist); gỡ block cross-đội.</t>
-  </si>
-  <si>
-    <t>Dùng CI/CD; env/secrets; logging/error tracking; deploy an toàn; tham gia oncall.</t>
-  </si>
-  <si>
-    <t>Cải thiện CI/CD, metrics/alerts, rollback; reliability xuyên stack.</t>
-  </si>
-  <si>
-    <t>Chuẩn hóa release/observability; playbooks; giảm MTTR; mentoring thực hành ops.</t>
-  </si>
-  <si>
-    <t>AI Agent xuyên stack cho scaffolding/refactor/tests/debug; kỹ thuật prompt; review cẩn thận.</t>
-  </si>
-  <si>
-    <t>Prompt/workflow tái sử dụng; AI cho debugging/review; đo impact.</t>
-  </si>
-  <si>
-    <t>Dẫn kỹ thuật AI; đào tạo đội; tự động hóa công việc end-to-end an toàn có governance.</t>
-  </si>
-  <si>
-    <t>Gợi ý: dùng nút +/- (Outline) để thu gọn/mở rộng theo từng Vai trò. Cấp độ 1: Làm tốt phần việc kỹ thuật của mình | Cấp độ 2: Giải quyết bài toán xuyên hệ thống | Cấp độ 3: Định hướng, tạo chuẩn, scale team</t>
-  </si>
-  <si>
-    <t>Quản lý scope/risk chủ động; phối hợp các bộ phận; giảm rework nhờ specs/docs tốt hơn.</t>
-  </si>
-  <si>
-    <t>Cải tiến quy trình bàn giao công việc trong team (tiêu chí hoàn thành, checklist rà soát); xử lý các điểm nghẽn phối hợp giữa team; nâng cao tính dự báo và kiểm soát tiến độ.</t>
+    <t>MÔ TẢ NĂNG LỰC THEO VAI TRÒ</t>
+  </si>
+  <si>
+    <t>Định hướng kiến trúc hệ thống có khả năng mở rộng; chủ động ngăn ngừa rủi ro và lỗi hệ thống; dẫn dắt cải tiến kỹ thuật lớn và hỗ trợ nâng cao năng lực đội ngũ.</t>
+  </si>
+  <si>
+    <t>Bàn giao công việc ổn định; biết tách công việc thành các đầu việc rõ ràng; chịu trách nhiệm xử lý lỗi đến khi hoàn tất; chủ động báo sớm các rủi ro phát sinh.</t>
+  </si>
+  <si>
+    <t>Chủ động quản lý phạm vi và rủi ro công việc; phối hợp hiệu quả với các bộ phận liên quan; giảm phát sinh làm lại nhờ yêu cầu và tài liệu được chuẩn bị rõ ràng.</t>
+  </si>
+  <si>
+    <t>Cải tiến quy trình bàn giao công việc trong đội (tiêu chí hoàn thành, danh sách rà soát); xử lý các điểm nghẽn trong phối hợp giữa các nhóm; nâng cao khả năng dự báo và kiểm soát tiến độ chung.</t>
+  </si>
+  <si>
+    <t>Thực hiện quy trình tích hợp và triển khai tự động; hiểu và sử dụng đúng cấu hình môi trường, thông tin bảo mật; theo dõi nhật ký và lỗi hệ thống; tham gia trực xử lý sự cố khi cần.</t>
+  </si>
+  <si>
+    <t>Chủ động cải thiện quy trình triển khai (tối ưu hiệu năng, kiểm soát chất lượng); bổ sung theo dõi chỉ số và cảnh báo; thực hiện phương án quay lui khi có sự cố; nâng cao độ ổn định và rút ngắn thời gian khắc phục lỗi.</t>
+  </si>
+  <si>
+    <t>Chuẩn hóa quy trình phát hành và giám sát hệ thống; xây dựng hướng dẫn vận hành và xử lý sự cố; chủ trì phân tích nguyên nhân sau sự cố; hướng dẫn và nâng cao năng lực vận hành cho đội ngũ.</t>
+  </si>
+  <si>
+    <t>Xây dựng mẫu yêu cầu và quy trình làm việc có thể tái sử dụng; dùng AI để hỗ trợ rà soát và tìm lỗi; theo dõi hiệu quả bằng các chỉ số như thời gian hoàn thành và tỷ lệ lỗi phát sinh.</t>
+  </si>
+  <si>
+    <t>Dẫn dắt việc áp dụng AI trong kỹ thuật một cách có kiểm soát; đào tạo và hướng dẫn đội ngũ; tự động hóa các công việc lặp lại theo nguyên tắc an toàn, phân quyền và tuân thủ quy định nội bộ.</t>
+  </si>
+  <si>
+    <t>Sử dụng AI Agent để hỗ trợ code, chỉnh sửa code, viết kiểm thử và tìm lỗi; biết đặt yêu cầu rõ ràng; luôn kiểm tra lại kết quả trước khi áp dụng.</t>
+  </si>
+  <si>
+    <t>Tự xây dựng luồng trải nghiệm và đặc tả giao diện; đảm bảo tính nhất quán về hình ảnh; bàn giao thiết kế rõ ràng để đội triển khai chính xác.</t>
+  </si>
+  <si>
+    <t>Cải thiện khả năng sử dụng dựa trên nghiên cứu và đánh giá trải nghiệm; phát triển và mở rộng hệ thống thiết kế; giảm phát sinh làm lại nhờ đặc tả thiết kế rõ ràng.</t>
+  </si>
+  <si>
+    <t>Định hướng thiết kế tổng thể; tạo ra tác động trải nghiệm người dùng có thể đo lường; quản trị và chuẩn hóa hệ thống thiết kế; hướng dẫn và kết nối các đội cùng áp dụng.</t>
+  </si>
+  <si>
+    <t>Bàn giao công việc ổn định; xác định rõ phạm vi; lặp lại thiết kế kịp thời; phối hợp sớm với các bên triển khai để thống nhất ràng buộc.</t>
+  </si>
+  <si>
+    <t>Quản lý các lựa chọn và đánh đổi trong thiết kế; chuẩn bị phương án thay thế; ghi nhận rõ các quyết định; giảm phát sinh làm lại thông qua rà soát thiết kế.</t>
+  </si>
+  <si>
+    <t>Nâng chuẩn bàn giao thiết kế (tiêu chí hoàn thành, danh sách rà soát); tháo gỡ các vướng mắc phối hợp giữa các đội; nâng cao khả năng dự báo và kiểm soát tiến độ.</t>
+  </si>
+  <si>
+    <t>Làm việc với môi trường preview và staging; sử dụng nhất quán các thành phần và chuẩn thiết kế; xây dựng đặc tả phù hợp với khả năng triển khai.</t>
+  </si>
+  <si>
+    <t>Thúc đẩy áp dụng chuẩn thành phần thiết kế; cải thiện tự động hóa bàn giao thiết kế–triển khai; giảm lỗi tích hợp và công việc làm lại.</t>
+  </si>
+  <si>
+    <t>Dẫn dắt chuẩn hóa quy trình thiết kế–triển khai với đội phát triển; xây dựng hướng dẫn và các thực hành tốt cho toàn đội.</t>
+  </si>
+  <si>
+    <t>Sử dụng AI để hỗ trợ xây dựng khung thiết kế, nội dung trải nghiệm và phương án thiết kế; biết đặt yêu cầu phù hợp; kiểm tra và đối chiếu với hệ thống thiết kế hiện có.</t>
+  </si>
+  <si>
+    <t>Xây dựng thư viện yêu cầu AI có thể tái sử dụng; tăng tốc tổng hợp nghiên cứu; theo dõi tác động của AI đến thời gian thực hiện và mức độ làm lại.</t>
+  </si>
+  <si>
+    <t>Dẫn dắt việc áp dụng AI trong thiết kế một cách an toàn và có kiểm soát; đào tạo đội ngũ; tự động hóa các công việc lặp lại theo quy định và chuẩn quản trị.</t>
+  </si>
+  <si>
+    <t>Gợi ý: dùng nút +/- (Outline) để thu gọn/mở rộng theo từng Vai trò. Cấp độ 1 (Thực thi – phối hợp): Làm tốt phần việc kỹ thuật của mình | Cấp độ 2 (Chủ động – cải tiến): Giải quyết bài toán xuyên hệ thống | Cấp độ 3 (Chuẩn hoá – dẫn dắt): Định hướng, tạo chuẩn, mở rộng</t>
+  </si>
+  <si>
+    <t>Tự triển khai tính năng giao diện từ đầu đến cuối (giao diện, trạng thái, tích hợp dữ liệu); xử lý các tình huống phát sinh; viết mã rõ ràng, dễ bảo trì.</t>
+  </si>
+  <si>
+    <t>Cải thiện hiệu năng và khả năng truy cập của giao diện; xây dựng thành phần dùng lại; nâng cao kiến trúc và kiểm thử để tăng độ ổn định.</t>
+  </si>
+  <si>
+    <t>Định hướng kỹ thuật frontend; dẫn dắt các thay đổi lớn để giảm rủi ro; hướng dẫn đội ngũ; chủ động ngăn ngừa lỗi ảnh hưởng diện rộng trên giao diện.</t>
+  </si>
+  <si>
+    <t>Bàn giao công việc ổn định; chịu trách nhiệm xử lý lỗi đến khi hoàn tất; phối hợp sớm với backend và thiết kế; chủ động báo rủi ro.</t>
+  </si>
+  <si>
+    <t>Quản lý các lựa chọn và đánh đổi về trải nghiệm người dùng; giảm phát sinh làm lại; nâng chất lượng bàn giao bằng đặc tả, minh chứng và tài liệu rõ ràng.</t>
+  </si>
+  <si>
+    <t>Nâng chuẩn bàn giao và rà soát (chuẩn thành phần, danh sách rà soát); tháo gỡ vướng mắc phối hợp giữa các đội; nâng cao khả năng dự báo và kiểm soát tiến độ.</t>
+  </si>
+  <si>
+    <t>Sử dụng thành thạo quy trình tích hợp và triển khai; quản lý cấu hình môi trường; theo dõi lỗi phía người dùng; giữ bản phát hành gọn và ổn định.</t>
+  </si>
+  <si>
+    <t>Cải thiện quy trình triển khai (tối ưu tốc độ, kiểm soát chất lượng); giảm kích thước và thời gian tải; có phương án quay lui khi sự cố; nâng cao độ ổn định.</t>
+  </si>
+  <si>
+    <t>Chuẩn hóa phát hành và giám sát cho frontend; xây dựng hướng dẫn xử lý sự cố; hướng dẫn đội ngũ thực hành vận hành; giảm lỗi phía người dùng và rút ngắn thời gian khắc phục.</t>
+  </si>
+  <si>
+    <t>Sử dụng AI để hỗ trợ tạo khung code, chỉnh sửa code, viết kiểm thử và tìm lỗi; biết đặt yêu cầu rõ ràng; luôn kiểm tra lại trước khi áp dụng.</t>
+  </si>
+  <si>
+    <t>Xây dựng mẫu yêu cầu AI có thể tái sử dụng (thành phần, khả năng truy cập, kiểm thử); dùng AI hỗ trợ rà soát và cải tiến mã; theo dõi hiệu quả bằng các chỉ số phù hợp.</t>
+  </si>
+  <si>
+    <t>Dẫn dắt việc áp dụng AI trong frontend theo quy chuẩn; đào tạo đội ngũ; tự động hóa các công việc lặp lại một cách an toàn và có kiểm soát.</t>
+  </si>
+  <si>
+    <t>Tự triển khai tính năng từ đầu đến cuối (giao diện, xử lý dữ liệu, lưu trữ); đảm bảo chất lượng cơ bản; viết kiểm thử cần thiết; xử lý các tình huống lỗi phát sinh.</t>
+  </si>
+  <si>
+    <t>Phân định rõ trách nhiệm giữa backend và frontend; cải thiện hiệu năng và an toàn hệ thống; thực hiện tái cấu trúc có kiểm soát; xây dựng kiểm thử vững chắc hơn.</t>
+  </si>
+  <si>
+    <t>Định hướng kỹ thuật end-to-end; chủ động ngăn ngừa rủi ro và lỗi hệ thống; hướng dẫn đội ngũ; dẫn dắt các đợt tái cấu trúc và chuyển đổi hệ thống lớn một cách an toàn.</t>
+  </si>
+  <si>
+    <t>Chịu trách nhiệm toàn bộ tính năng từ đầu đến cuối; đảm bảo vận hành ổn định; chủ động báo rủi ro; xử lý triệt để vấn đề đến khi hoàn tất.</t>
+  </si>
+  <si>
+    <t>Quản lý phạm vi và rủi ro công việc; trao đổi và thống nhất các đánh đổi kỹ thuật; giảm phát sinh làm lại; cải thiện chất lượng tài liệu và bàn giao.</t>
+  </si>
+  <si>
+    <t>Nâng cao khả năng dự báo; xây dựng và áp dụng các chuẩn chung (tiêu chí hoàn thành, danh sách rà soát); tháo gỡ vướng mắc trong phối hợp giữa các đội.</t>
+  </si>
+  <si>
+    <t>Sử dụng quy trình tích hợp và triển khai tự động; quản lý cấu hình và thông tin bảo mật; theo dõi lỗi và nhật ký hệ thống; triển khai an toàn và tham gia trực xử lý sự cố.</t>
+  </si>
+  <si>
+    <t>Cải thiện quy trình triển khai; bổ sung theo dõi chỉ số và cảnh báo; có phương án quay lui khi cần; nâng cao độ ổn định trên toàn bộ hệ thống.</t>
+  </si>
+  <si>
+    <t>Chuẩn hóa phát hành và giám sát hệ thống; xây dựng hướng dẫn vận hành và xử lý sự cố; giảm thời gian khắc phục lỗi; hướng dẫn đội ngũ thực hành vận hành hiệu quả.</t>
+  </si>
+  <si>
+    <t>Sử dụng AI hỗ trợ toàn bộ chuỗi phát triển (tạo khung, chỉnh sửa code, kiểm thử, tìm lỗi); biết đặt yêu cầu phù hợp; luôn rà soát kỹ kết quả trước khi áp dụng.</t>
+  </si>
+  <si>
+    <t>Xây dựng mẫu yêu cầu và quy trình làm việc với AI có thể tái sử dụng; dùng AI hỗ trợ rà soát và tìm lỗi; theo dõi tác động đến thời gian thực hiện và chất lượng.</t>
+  </si>
+  <si>
+    <t>Dẫn dắt việc áp dụng AI trong phát triển end-to-end một cách an toàn và có kiểm soát; đào tạo đội ngũ; tự động hóa các công việc xuyên suốt theo chuẩn quản trị.</t>
   </si>
 </sst>
 </file>
@@ -554,7 +554,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -589,6 +589,9 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -596,15 +599,15 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -617,10 +620,10 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -973,28 +976,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-      <c r="E3" s="13"/>
-      <c r="F3" s="13"/>
-      <c r="G3" s="13"/>
-      <c r="H3" s="13"/>
+      <c r="B3" s="14"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="14"/>
+      <c r="H3" s="14"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -1616,31 +1619,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
     </row>
     <row r="3" spans="1:5" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="12"/>
-      <c r="C3" s="13"/>
+      <c r="B3" s="13"/>
+      <c r="C3" s="14"/>
       <c r="D3" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="12"/>
+      <c r="E3" s="13"/>
     </row>
     <row r="4" spans="1:5" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="12"/>
-      <c r="C4" s="13"/>
+      <c r="B4" s="13"/>
+      <c r="C4" s="14"/>
       <c r="D4" s="5" t="s">
         <v>18</v>
       </c>
@@ -1734,19 +1737,19 @@
       <c r="E11" s="7"/>
     </row>
     <row r="13" spans="1:5" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="15" t="s">
+      <c r="A13" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="B13" s="13"/>
-      <c r="C13" s="13"/>
-      <c r="D13" s="13"/>
-      <c r="E13" s="13"/>
+      <c r="B13" s="14"/>
+      <c r="C13" s="14"/>
+      <c r="D13" s="14"/>
+      <c r="E13" s="14"/>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B14" s="20" t="s">
+      <c r="B14" s="21" t="s">
         <v>31</v>
       </c>
       <c r="C14" s="17"/>
@@ -1757,7 +1760,7 @@
       <c r="A15" s="8">
         <v>1</v>
       </c>
-      <c r="B15" s="16" t="s">
+      <c r="B15" s="20" t="s">
         <v>32</v>
       </c>
       <c r="C15" s="17"/>
@@ -1768,7 +1771,7 @@
       <c r="A16" s="8">
         <v>2</v>
       </c>
-      <c r="B16" s="16" t="s">
+      <c r="B16" s="20" t="s">
         <v>33</v>
       </c>
       <c r="C16" s="17"/>
@@ -1779,7 +1782,7 @@
       <c r="A17" s="8">
         <v>3</v>
       </c>
-      <c r="B17" s="16" t="s">
+      <c r="B17" s="20" t="s">
         <v>34</v>
       </c>
       <c r="C17" s="17"/>
@@ -1790,7 +1793,7 @@
       <c r="A18" s="8">
         <v>4</v>
       </c>
-      <c r="B18" s="16" t="s">
+      <c r="B18" s="20" t="s">
         <v>35</v>
       </c>
       <c r="C18" s="17"/>
@@ -1801,7 +1804,7 @@
       <c r="A19" s="8">
         <v>5</v>
       </c>
-      <c r="B19" s="16" t="s">
+      <c r="B19" s="20" t="s">
         <v>36</v>
       </c>
       <c r="C19" s="17"/>
@@ -1809,13 +1812,13 @@
       <c r="E19" s="18"/>
     </row>
     <row r="21" spans="1:5" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="15" t="s">
+      <c r="A21" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="B21" s="13"/>
-      <c r="C21" s="13"/>
-      <c r="D21" s="13"/>
-      <c r="E21" s="13"/>
+      <c r="B21" s="14"/>
+      <c r="C21" s="14"/>
+      <c r="D21" s="14"/>
+      <c r="E21" s="14"/>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
@@ -1824,7 +1827,7 @@
       <c r="B22" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C22" s="20" t="s">
+      <c r="C22" s="21" t="s">
         <v>39</v>
       </c>
       <c r="D22" s="17"/>
@@ -1837,7 +1840,7 @@
       <c r="B23" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="C23" s="19" t="s">
+      <c r="C23" s="16" t="s">
         <v>42</v>
       </c>
       <c r="D23" s="17"/>
@@ -1850,7 +1853,7 @@
       <c r="B24" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C24" s="19" t="s">
+      <c r="C24" s="16" t="s">
         <v>45</v>
       </c>
       <c r="D24" s="17"/>
@@ -1863,7 +1866,7 @@
       <c r="B25" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="C25" s="19" t="s">
+      <c r="C25" s="16" t="s">
         <v>48</v>
       </c>
       <c r="D25" s="17"/>
@@ -1876,7 +1879,7 @@
       <c r="B26" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="C26" s="19" t="s">
+      <c r="C26" s="16" t="s">
         <v>51</v>
       </c>
       <c r="D26" s="17"/>
@@ -1884,6 +1887,12 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A21:E21"/>
+    <mergeCell ref="B17:E17"/>
+    <mergeCell ref="B18:E18"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="E3"/>
     <mergeCell ref="C26:E26"/>
     <mergeCell ref="A13:E13"/>
     <mergeCell ref="B19:E19"/>
@@ -1895,12 +1904,6 @@
     <mergeCell ref="C22:E22"/>
     <mergeCell ref="B16:E16"/>
     <mergeCell ref="B15:E15"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A21:E21"/>
-    <mergeCell ref="B17:E17"/>
-    <mergeCell ref="B18:E18"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="E3"/>
   </mergeCells>
   <conditionalFormatting sqref="C7:C10">
     <cfRule type="cellIs" dxfId="8" priority="1" operator="equal">
@@ -1952,41 +1955,41 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+    </row>
+    <row r="2" spans="1:4" ht="36.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="24" t="s">
+        <v>86</v>
+      </c>
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+    </row>
+    <row r="4" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-    </row>
-    <row r="2" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="23" t="s">
-        <v>108</v>
-      </c>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
-    </row>
-    <row r="4" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="22" t="s">
-        <v>53</v>
-      </c>
-      <c r="B4" s="13"/>
-      <c r="C4" s="13"/>
-      <c r="D4" s="13"/>
+      <c r="B4" s="14"/>
+      <c r="C4" s="14"/>
+      <c r="D4" s="14"/>
     </row>
     <row r="5" spans="1:4" ht="19.95" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
         <v>19</v>
       </c>
       <c r="B5" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="C5" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="C5" s="9" t="s">
+      <c r="D5" s="9" t="s">
         <v>55</v>
-      </c>
-      <c r="D5" s="9" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="79.95" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
@@ -1994,289 +1997,289 @@
         <v>24</v>
       </c>
       <c r="B6" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="C6" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="C6" s="11" t="s">
-        <v>58</v>
-      </c>
-      <c r="D6" s="11" t="s">
-        <v>59</v>
+      <c r="D6" s="12" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="79.95" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A7" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="B7" s="11" t="s">
-        <v>60</v>
-      </c>
-      <c r="C7" s="24" t="s">
-        <v>109</v>
-      </c>
-      <c r="D7" s="24" t="s">
-        <v>110</v>
+      <c r="B7" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="D7" s="12" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="79.95" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A8" s="10" t="s">
-        <v>61</v>
-      </c>
-      <c r="B8" s="11" t="s">
-        <v>62</v>
-      </c>
-      <c r="C8" s="24" t="s">
-        <v>63</v>
-      </c>
-      <c r="D8" s="11" t="s">
-        <v>64</v>
+        <v>58</v>
+      </c>
+      <c r="B8" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="D8" s="12" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="79.95" customHeight="1" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.3">
       <c r="A9" s="10" t="s">
-        <v>65</v>
-      </c>
-      <c r="B9" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="C9" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="D9" s="11" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="22.05" customHeight="1" collapsed="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="22" t="s">
-        <v>69</v>
-      </c>
-      <c r="B11" s="13"/>
-      <c r="C11" s="13"/>
-      <c r="D11" s="13"/>
-    </row>
-    <row r="12" spans="1:4" ht="19.95" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+      <c r="B9" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="D9" s="12" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="23" t="s">
+        <v>60</v>
+      </c>
+      <c r="B11" s="14"/>
+      <c r="C11" s="14"/>
+      <c r="D11" s="14"/>
+    </row>
+    <row r="12" spans="1:4" ht="19.95" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A12" s="9" t="s">
         <v>19</v>
       </c>
       <c r="B12" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="C12" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="C12" s="9" t="s">
+      <c r="D12" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="D12" s="9" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="79.95" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="13" spans="1:4" ht="79.95" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A13" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="B13" s="11" t="s">
-        <v>70</v>
-      </c>
-      <c r="C13" s="11" t="s">
-        <v>71</v>
-      </c>
-      <c r="D13" s="11" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="79.95" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="B13" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="C13" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="D13" s="12" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="79.95" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A14" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="B14" s="11" t="s">
-        <v>73</v>
-      </c>
-      <c r="C14" s="11" t="s">
-        <v>74</v>
-      </c>
-      <c r="D14" s="11" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" ht="79.95" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="C14" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="D14" s="12" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="79.95" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A15" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="B15" s="12" t="s">
+        <v>80</v>
+      </c>
+      <c r="C15" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="D15" s="12" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="79.95" customHeight="1" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="B16" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="D16" s="12" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="23" t="s">
         <v>61</v>
       </c>
-      <c r="B15" s="11" t="s">
-        <v>76</v>
-      </c>
-      <c r="C15" s="11" t="s">
-        <v>77</v>
-      </c>
-      <c r="D15" s="11" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" ht="79.95" hidden="1" customHeight="1" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="10" t="s">
-        <v>65</v>
-      </c>
-      <c r="B16" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="C16" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="D16" s="11" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" ht="22.05" customHeight="1" collapsed="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="22" t="s">
-        <v>82</v>
-      </c>
-      <c r="B18" s="13"/>
-      <c r="C18" s="13"/>
-      <c r="D18" s="13"/>
-    </row>
-    <row r="19" spans="1:4" ht="19.95" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="B18" s="14"/>
+      <c r="C18" s="14"/>
+      <c r="D18" s="14"/>
+    </row>
+    <row r="19" spans="1:4" ht="19.95" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A19" s="9" t="s">
         <v>19</v>
       </c>
       <c r="B19" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="C19" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="C19" s="9" t="s">
+      <c r="D19" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="D19" s="9" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" ht="79.95" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="20" spans="1:4" ht="79.95" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A20" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="B20" s="11" t="s">
-        <v>83</v>
-      </c>
-      <c r="C20" s="11" t="s">
-        <v>84</v>
-      </c>
-      <c r="D20" s="11" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" ht="79.95" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="B20" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="C20" s="12" t="s">
+        <v>88</v>
+      </c>
+      <c r="D20" s="12" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="79.95" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A21" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="B21" s="11" t="s">
-        <v>86</v>
-      </c>
-      <c r="C21" s="11" t="s">
-        <v>87</v>
-      </c>
-      <c r="D21" s="11" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" ht="79.95" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="B21" s="12" t="s">
+        <v>90</v>
+      </c>
+      <c r="C21" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="D21" s="12" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="79.95" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A22" s="10" t="s">
-        <v>61</v>
-      </c>
-      <c r="B22" s="11" t="s">
-        <v>89</v>
-      </c>
-      <c r="C22" s="11" t="s">
-        <v>90</v>
-      </c>
-      <c r="D22" s="11" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" ht="79.95" hidden="1" customHeight="1" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.3">
+        <v>58</v>
+      </c>
+      <c r="B22" s="12" t="s">
+        <v>93</v>
+      </c>
+      <c r="C22" s="12" t="s">
+        <v>94</v>
+      </c>
+      <c r="D22" s="12" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="79.95" customHeight="1" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.3">
       <c r="A23" s="10" t="s">
-        <v>65</v>
-      </c>
-      <c r="B23" s="11" t="s">
-        <v>92</v>
-      </c>
-      <c r="C23" s="11" t="s">
-        <v>93</v>
-      </c>
-      <c r="D23" s="11" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" ht="22.05" customHeight="1" collapsed="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="22" t="s">
-        <v>95</v>
-      </c>
-      <c r="B25" s="13"/>
-      <c r="C25" s="13"/>
-      <c r="D25" s="13"/>
-    </row>
-    <row r="26" spans="1:4" ht="19.95" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+      <c r="B23" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="C23" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="D23" s="12" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="23" t="s">
+        <v>62</v>
+      </c>
+      <c r="B25" s="14"/>
+      <c r="C25" s="14"/>
+      <c r="D25" s="14"/>
+    </row>
+    <row r="26" spans="1:4" ht="19.95" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A26" s="9" t="s">
         <v>19</v>
       </c>
       <c r="B26" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="C26" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="C26" s="9" t="s">
+      <c r="D26" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="D26" s="9" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" ht="79.95" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="27" spans="1:4" ht="79.95" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A27" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="B27" s="11" t="s">
-        <v>96</v>
-      </c>
-      <c r="C27" s="11" t="s">
-        <v>97</v>
-      </c>
-      <c r="D27" s="11" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" ht="79.95" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="B27" s="12" t="s">
+        <v>99</v>
+      </c>
+      <c r="C27" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="D27" s="12" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="79.95" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A28" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="B28" s="11" t="s">
-        <v>99</v>
-      </c>
-      <c r="C28" s="11" t="s">
-        <v>100</v>
-      </c>
-      <c r="D28" s="11" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" ht="79.95" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="B28" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="C28" s="12" t="s">
+        <v>103</v>
+      </c>
+      <c r="D28" s="12" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" ht="79.95" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A29" s="10" t="s">
-        <v>61</v>
-      </c>
-      <c r="B29" s="11" t="s">
-        <v>102</v>
-      </c>
-      <c r="C29" s="11" t="s">
-        <v>103</v>
-      </c>
-      <c r="D29" s="11" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" ht="79.95" hidden="1" customHeight="1" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.3">
+        <v>58</v>
+      </c>
+      <c r="B29" s="12" t="s">
+        <v>105</v>
+      </c>
+      <c r="C29" s="12" t="s">
+        <v>106</v>
+      </c>
+      <c r="D29" s="12" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" ht="79.95" customHeight="1" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.3">
       <c r="A30" s="10" t="s">
-        <v>65</v>
-      </c>
-      <c r="B30" s="11" t="s">
-        <v>105</v>
-      </c>
-      <c r="C30" s="11" t="s">
-        <v>106</v>
-      </c>
-      <c r="D30" s="11" t="s">
-        <v>107</v>
+        <v>59</v>
+      </c>
+      <c r="B30" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="C30" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="D30" s="12" t="s">
+        <v>110</v>
       </c>
     </row>
   </sheetData>

</xml_diff>